<commit_message>
feat: complete Avalonia migration
</commit_message>
<xml_diff>
--- a/Excel/Label.xlsx
+++ b/Excel/Label.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source\AppPlayerMacro\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD676934-C533-463E-882D-7250DD7C193C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80832E5F-7875-4237-901B-E3EAB0D3F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7095" yWindow="975" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5190" yWindow="2490" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="203">
   <si>
     <t>Name</t>
   </si>
@@ -88,22 +88,13 @@
     <t>Preferences</t>
   </si>
   <si>
-    <t>EventType</t>
-  </si>
-  <si>
     <t>이벤트 타입</t>
   </si>
   <si>
-    <t>EventDataSet</t>
-  </si>
-  <si>
     <t>이벤트 데이터</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>TriggerList</t>
-  </si>
-  <si>
     <t>트리거 리스트</t>
   </si>
   <si>
@@ -153,33 +144,21 @@
     <t>중지</t>
   </si>
   <si>
-    <t>Setting</t>
-  </si>
-  <si>
     <t>Language</t>
   </si>
   <si>
     <t>언어</t>
   </si>
   <si>
-    <t>SavePath</t>
-  </si>
-  <si>
     <t>저장 경로</t>
   </si>
   <si>
     <t>전체 프로세싱 주기(ms)</t>
   </si>
   <si>
-    <t>Period(ms)</t>
-  </si>
-  <si>
     <t>아이템 딜레이(ms)</t>
   </si>
   <si>
-    <t>ItemDelay(ms)</t>
-  </si>
-  <si>
     <t>Similarity</t>
   </si>
   <si>
@@ -189,10 +168,6 @@
     <t>후(後) 작업 딜레이(ms)</t>
   </si>
   <si>
-    <t>AfterDelay(ms)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>이미지 검색 결과 표시</t>
   </si>
   <si>
@@ -272,9 +247,6 @@
     <t>바로 이동</t>
   </si>
   <si>
-    <t>ToNext</t>
-  </si>
-  <si>
     <t>패치 실패</t>
   </si>
   <si>
@@ -329,10 +301,6 @@
     <t>물리 클릭</t>
   </si>
   <si>
-    <t>Hard Click</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>관심영역 설정</t>
   </si>
   <si>
@@ -403,10 +371,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MacroMode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>KeyboardDelay(ms)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -469,19 +433,236 @@
     <t>StopOnParentImage</t>
   </si>
   <si>
-    <t>이미지 뷰어 보기</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Show Image Viewer</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>항목별 유사도</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Item Similarity</t>
+  </si>
+  <si>
+    <t>Event type</t>
+  </si>
+  <si>
+    <t>Input details</t>
+  </si>
+  <si>
+    <t>Events</t>
+  </si>
+  <si>
+    <t>설정</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>Save folder</t>
+  </si>
+  <si>
+    <t>Process interval (ms)</t>
+  </si>
+  <si>
+    <t>Event interval (ms)</t>
+  </si>
+  <si>
+    <t>Delay after event (ms)</t>
+  </si>
+  <si>
+    <t>Next event</t>
+  </si>
+  <si>
+    <t>Physical click</t>
+  </si>
+  <si>
+    <t>실행 모드</t>
+  </si>
+  <si>
+    <t>Execution mode</t>
+  </si>
+  <si>
+    <t>1067</t>
+  </si>
+  <si>
+    <t>앱 업데이트</t>
+  </si>
+  <si>
+    <t>Application update</t>
+  </si>
+  <si>
+    <t>1068</t>
+  </si>
+  <si>
+    <t>현재 버전</t>
+  </si>
+  <si>
+    <t>Current version</t>
+  </si>
+  <si>
+    <t>1069</t>
+  </si>
+  <si>
+    <t>최신 정식 버전</t>
+  </si>
+  <si>
+    <t>Latest stable version</t>
+  </si>
+  <si>
+    <t>1070</t>
+  </si>
+  <si>
+    <t>업데이트 확인</t>
+  </si>
+  <si>
+    <t>Check for updates</t>
+  </si>
+  <si>
+    <t>1071</t>
+  </si>
+  <si>
+    <t>업데이트 후 재시작</t>
+  </si>
+  <si>
+    <t>Update and restart</t>
+  </si>
+  <si>
+    <t>1072</t>
+  </si>
+  <si>
+    <t>릴리스 열기</t>
+  </si>
+  <si>
+    <t>Open releases</t>
+  </si>
+  <si>
+    <t>1073</t>
+  </si>
+  <si>
+    <t>이미지</t>
+  </si>
+  <si>
+    <t>Image</t>
+  </si>
+  <si>
+    <t>1074</t>
+  </si>
+  <si>
+    <t>번호</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>1075</t>
+  </si>
+  <si>
+    <t>프로세스</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>1076</t>
+  </si>
+  <si>
+    <t>실행 상태</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>1077</t>
+  </si>
+  <si>
+    <t>위로 이동</t>
+  </si>
+  <si>
+    <t>Move up</t>
+  </si>
+  <si>
+    <t>1078</t>
+  </si>
+  <si>
+    <t>아래로 이동</t>
+  </si>
+  <si>
+    <t>Move down</t>
+  </si>
+  <si>
+    <t>1079</t>
+  </si>
+  <si>
+    <t>입력 설정</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>1080</t>
+  </si>
+  <si>
+    <t>실행 설정</t>
+  </si>
+  <si>
+    <t>Execution</t>
+  </si>
+  <si>
+    <t>1081</t>
+  </si>
+  <si>
+    <t>화면 설정</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>1082</t>
+  </si>
+  <si>
+    <t>아직 등록된 이벤트가 없습니다.</t>
+  </si>
+  <si>
+    <t>No events yet.</t>
+  </si>
+  <si>
+    <t>1083</t>
+  </si>
+  <si>
+    <t>프로세스를 선택하고 추가 버튼을 눌러 첫 이미지를 캡처하세요.</t>
+  </si>
+  <si>
+    <t>Select a process and choose Add to capture your first image.</t>
+  </si>
+  <si>
+    <t>1084</t>
+  </si>
+  <si>
+    <t>대상 창을 화면에 표시해 두세요. 창을 활성화하고 실제 마우스 커서를 움직여 클릭합니다. 같은 이미지 드래그와는 함께 사용할 수 없습니다.</t>
+  </si>
+  <si>
+    <t>Keep the target window visible. This activates the window and moves your mouse cursor to click. Not available with same-image dragging.</t>
+  </si>
+  <si>
+    <t>1085</t>
+  </si>
+  <si>
+    <t>전체 선택</t>
+  </si>
+  <si>
+    <t>Select all</t>
+  </si>
+  <si>
+    <t>1086</t>
+  </si>
+  <si>
+    <t>실행할 프로세스와 이벤트를 선택하세요.</t>
+  </si>
+  <si>
+    <t>Choose a process and the events to run.</t>
+  </si>
+  <si>
+    <t>로그 폴더 열기</t>
+  </si>
+  <si>
+    <t>Open log folder</t>
   </si>
 </sst>
 </file>
@@ -856,7 +1037,7 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -895,7 +1076,7 @@
         <v>1004</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
@@ -923,12 +1104,10 @@
         <v>1006</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Event type</t>
-        </is>
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -939,12 +1118,10 @@
         <v>1007</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Input details</t>
-        </is>
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -955,12 +1132,10 @@
         <v>1008</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -971,10 +1146,10 @@
         <v>1009</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -985,10 +1160,10 @@
         <v>1010</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -999,10 +1174,10 @@
         <v>1011</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1013,10 +1188,10 @@
         <v>1012</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -1027,10 +1202,10 @@
         <v>1013</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -1041,10 +1216,10 @@
         <v>1014</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1055,10 +1230,10 @@
         <v>1015</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1068,15 +1243,11 @@
       <c r="B18">
         <v>1016</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>설정</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
+      <c r="C18" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1087,10 +1258,10 @@
         <v>1017</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D19" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1101,10 +1272,10 @@
         <v>1018</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1115,12 +1286,10 @@
         <v>1019</v>
       </c>
       <c r="C21" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Save folder</t>
-        </is>
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1131,12 +1300,10 @@
         <v>1020</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Process interval (ms)</t>
-        </is>
+        <v>40</v>
+      </c>
+      <c r="D22" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1147,12 +1314,10 @@
         <v>1021</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Event interval (ms)</t>
-        </is>
+        <v>41</v>
+      </c>
+      <c r="D23" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1163,10 +1328,10 @@
         <v>1022</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1177,12 +1342,10 @@
         <v>1023</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Delay after event (ms)</t>
-        </is>
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1193,10 +1356,10 @@
         <v>1024</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1207,10 +1370,10 @@
         <v>1025</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1221,10 +1384,10 @@
         <v>1026</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -1235,10 +1398,10 @@
         <v>1027</v>
       </c>
       <c r="C29" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D29" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1246,13 +1409,13 @@
         <v>1028</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D30" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -1263,7 +1426,7 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
         <v>1</v>
@@ -1274,13 +1437,13 @@
         <v>1030</v>
       </c>
       <c r="B32" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -1288,13 +1451,13 @@
         <v>1031</v>
       </c>
       <c r="B33" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C33" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="D33" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1305,10 +1468,10 @@
         <v>1032</v>
       </c>
       <c r="C34" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D34" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -1319,10 +1482,10 @@
         <v>1033</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D35" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -1333,10 +1496,10 @@
         <v>1034</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -1347,10 +1510,10 @@
         <v>1035</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D37" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
@@ -1361,10 +1524,10 @@
         <v>1036</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D38" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
@@ -1375,10 +1538,10 @@
         <v>1037</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D39" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -1389,10 +1552,10 @@
         <v>1038</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D40" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -1403,12 +1566,10 @@
         <v>1039</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Next event</t>
-        </is>
+        <v>70</v>
+      </c>
+      <c r="D41" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
@@ -1419,10 +1580,10 @@
         <v>1040</v>
       </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D42" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
@@ -1433,10 +1594,10 @@
         <v>1041</v>
       </c>
       <c r="C43" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
@@ -1447,10 +1608,10 @@
         <v>1042</v>
       </c>
       <c r="C44" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="D44" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
@@ -1461,10 +1622,10 @@
         <v>1043</v>
       </c>
       <c r="C45" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D45" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -1475,10 +1636,10 @@
         <v>1044</v>
       </c>
       <c r="C46" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D46" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
@@ -1489,10 +1650,10 @@
         <v>1045</v>
       </c>
       <c r="C47" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="D47" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
@@ -1503,10 +1664,10 @@
         <v>1046</v>
       </c>
       <c r="C48" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="D48" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -1517,10 +1678,10 @@
         <v>1047</v>
       </c>
       <c r="C49" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="D49" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
@@ -1531,12 +1692,10 @@
         <v>1048</v>
       </c>
       <c r="C50" t="s">
-        <v>97</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Physical click</t>
-        </is>
+        <v>88</v>
+      </c>
+      <c r="D50" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
@@ -1547,10 +1706,10 @@
         <v>1049</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D51" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
@@ -1561,10 +1720,10 @@
         <v>1050</v>
       </c>
       <c r="C52" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D52" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
@@ -1575,10 +1734,10 @@
         <v>1051</v>
       </c>
       <c r="C53" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D53" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
@@ -1589,10 +1748,10 @@
         <v>1052</v>
       </c>
       <c r="C54" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D54" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -1603,10 +1762,10 @@
         <v>1053</v>
       </c>
       <c r="C55" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="D55" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="17.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -1617,10 +1776,10 @@
         <v>1054</v>
       </c>
       <c r="C56" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D56" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -1631,10 +1790,10 @@
         <v>1055</v>
       </c>
       <c r="C57" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D57" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
@@ -1645,10 +1804,10 @@
         <v>1056</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D58" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
@@ -1658,15 +1817,11 @@
       <c r="B59">
         <v>1057</v>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>실행 모드</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Execution mode</t>
-        </is>
+      <c r="C59" t="s">
+        <v>139</v>
+      </c>
+      <c r="D59" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
@@ -1677,10 +1832,10 @@
         <v>1058</v>
       </c>
       <c r="C60" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D60" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
@@ -1691,10 +1846,10 @@
         <v>1059</v>
       </c>
       <c r="C61" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="D61" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
@@ -1705,10 +1860,10 @@
         <v>1060</v>
       </c>
       <c r="C62" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D62" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
@@ -1719,10 +1874,10 @@
         <v>1061</v>
       </c>
       <c r="C63" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D63" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
@@ -1733,10 +1888,10 @@
         <v>1062</v>
       </c>
       <c r="C64" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="D64" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
@@ -1747,10 +1902,10 @@
         <v>1063</v>
       </c>
       <c r="C65" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D65" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
@@ -1761,438 +1916,318 @@
         <v>1064</v>
       </c>
       <c r="C66" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="D66" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="B67">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C67" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="D67" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>1066</v>
-      </c>
-      <c r="B68">
-        <v>1066</v>
+        <v>1067</v>
+      </c>
+      <c r="B68" t="s">
+        <v>141</v>
       </c>
       <c r="C68" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D68" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>1067</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1067</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>앱 업데이트</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Application update</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
+        <v>1068</v>
+      </c>
+      <c r="B69" t="s">
+        <v>144</v>
+      </c>
+      <c r="C69" t="s">
+        <v>145</v>
+      </c>
+      <c r="D69" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>1068</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1068</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>현재 버전</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Current version</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
+        <v>1069</v>
+      </c>
+      <c r="B70" t="s">
+        <v>147</v>
+      </c>
+      <c r="C70" t="s">
+        <v>148</v>
+      </c>
+      <c r="D70" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>1069</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>1069</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>최신 정식 버전</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Latest stable version</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
+        <v>1070</v>
+      </c>
+      <c r="B71" t="s">
+        <v>150</v>
+      </c>
+      <c r="C71" t="s">
+        <v>151</v>
+      </c>
+      <c r="D71" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>1070</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1070</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>업데이트 확인</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Check for updates</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
+        <v>1071</v>
+      </c>
+      <c r="B72" t="s">
+        <v>153</v>
+      </c>
+      <c r="C72" t="s">
+        <v>154</v>
+      </c>
+      <c r="D72" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>1071</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>1071</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>업데이트 후 재시작</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Update and restart</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
+        <v>1072</v>
+      </c>
+      <c r="B73" t="s">
+        <v>156</v>
+      </c>
+      <c r="C73" t="s">
+        <v>157</v>
+      </c>
+      <c r="D73" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>1072</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>1072</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>릴리스 열기</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Open releases</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
+        <v>1073</v>
+      </c>
+      <c r="B74" t="s">
+        <v>159</v>
+      </c>
+      <c r="C74" t="s">
+        <v>160</v>
+      </c>
+      <c r="D74" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75">
-        <v>1073</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>1073</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>이미지</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Image</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
+        <v>1074</v>
+      </c>
+      <c r="B75" t="s">
+        <v>162</v>
+      </c>
+      <c r="C75" t="s">
+        <v>163</v>
+      </c>
+      <c r="D75" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>1074</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>1074</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>번호</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Index</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
+        <v>1075</v>
+      </c>
+      <c r="B76" t="s">
+        <v>165</v>
+      </c>
+      <c r="C76" t="s">
+        <v>166</v>
+      </c>
+      <c r="D76" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>1075</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>1075</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>프로세스</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Process</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
+        <v>1076</v>
+      </c>
+      <c r="B77" t="s">
+        <v>168</v>
+      </c>
+      <c r="C77" t="s">
+        <v>169</v>
+      </c>
+      <c r="D77" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>1076</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>1076</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>실행 상태</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
+        <v>1077</v>
+      </c>
+      <c r="B78" t="s">
+        <v>171</v>
+      </c>
+      <c r="C78" t="s">
+        <v>172</v>
+      </c>
+      <c r="D78" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>1077</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>1077</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>위로 이동</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Move up</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
+        <v>1078</v>
+      </c>
+      <c r="B79" t="s">
+        <v>174</v>
+      </c>
+      <c r="C79" t="s">
+        <v>175</v>
+      </c>
+      <c r="D79" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>1078</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>1078</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>아래로 이동</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Move down</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
+        <v>1079</v>
+      </c>
+      <c r="B80" t="s">
+        <v>177</v>
+      </c>
+      <c r="C80" t="s">
+        <v>178</v>
+      </c>
+      <c r="D80" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81">
-        <v>1079</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>1079</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>입력 설정</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
+        <v>1080</v>
+      </c>
+      <c r="B81" t="s">
+        <v>180</v>
+      </c>
+      <c r="C81" t="s">
+        <v>181</v>
+      </c>
+      <c r="D81" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82">
-        <v>1080</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>1080</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>실행 설정</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Execution</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
+        <v>1081</v>
+      </c>
+      <c r="B82" t="s">
+        <v>183</v>
+      </c>
+      <c r="C82" t="s">
+        <v>184</v>
+      </c>
+      <c r="D82" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>1081</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>1081</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>화면 설정</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
+        <v>1082</v>
+      </c>
+      <c r="B83" t="s">
+        <v>186</v>
+      </c>
+      <c r="C83" t="s">
+        <v>187</v>
+      </c>
+      <c r="D83" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>1082</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>1082</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>아직 등록된 이벤트가 없습니다.</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>No events yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
+        <v>1083</v>
+      </c>
+      <c r="B84" t="s">
+        <v>189</v>
+      </c>
+      <c r="C84" t="s">
+        <v>190</v>
+      </c>
+      <c r="D84" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>1083</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>1083</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>프로세스를 선택하고 추가 버튼을 눌러 첫 이미지를 캡처하세요.</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Select a process and choose Add to capture your first image.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
+        <v>1084</v>
+      </c>
+      <c r="B85" t="s">
+        <v>192</v>
+      </c>
+      <c r="C85" t="s">
+        <v>193</v>
+      </c>
+      <c r="D85" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86">
-        <v>1084</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>1084</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>대상 창을 화면에 표시해 두세요. 창을 활성화하고 실제 마우스 커서를 움직여 클릭합니다. 같은 이미지 드래그와는 함께 사용할 수 없습니다.</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Keep the target window visible. This activates the window and moves your mouse cursor to click. Not available with same-image dragging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
+        <v>1085</v>
+      </c>
+      <c r="B86" t="s">
+        <v>195</v>
+      </c>
+      <c r="C86" t="s">
+        <v>196</v>
+      </c>
+      <c r="D86" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>1085</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>1085</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>전체 선택</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Select all</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
+        <v>1086</v>
+      </c>
+      <c r="B87" t="s">
+        <v>198</v>
+      </c>
+      <c r="C87" t="s">
+        <v>199</v>
+      </c>
+      <c r="D87" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88">
-        <v>1086</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>1086</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>실행할 프로세스와 이벤트를 선택하세요.</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Choose a process and the events to run.</t>
-        </is>
+        <v>1087</v>
+      </c>
+      <c r="B88">
+        <v>1087</v>
+      </c>
+      <c r="C88" t="s">
+        <v>201</v>
+      </c>
+      <c r="D88" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>